<commit_message>
changed path to remote repo folder names
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1017" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97B54914-1322-48B8-A520-41E5FF84C1A0}"/>
+  <xr:revisionPtr revIDLastSave="1019" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABBB021E-7055-4459-802D-1170FE4F6DF1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="1695" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,9 +116,6 @@
     <t>072925</t>
   </si>
   <si>
-    <t>Experimental data/MFM cal July 29/</t>
-  </si>
-  <si>
     <t>MFM-cal-Jul29-2025.dat</t>
   </si>
   <si>
@@ -192,6 +189,9 @@
   </si>
   <si>
     <t>GMT-4</t>
+  </si>
+  <si>
+    <t>data/BP-CAL-250729/</t>
   </si>
 </sst>
 </file>
@@ -641,27 +641,27 @@
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>25</v>
@@ -686,27 +686,27 @@
         <v>1</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>25</v>
@@ -731,27 +731,27 @@
         <v>1</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>25</v>
@@ -778,27 +778,27 @@
         <v>1</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>25</v>
@@ -825,27 +825,27 @@
         <v>1</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>25</v>
@@ -872,27 +872,27 @@
         <v>1</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>25</v>
@@ -919,27 +919,27 @@
         <v>1</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>25</v>
@@ -966,27 +966,27 @@
         <v>1</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>25</v>
@@ -1013,27 +1013,27 @@
         <v>1</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>25</v>
@@ -1060,27 +1060,27 @@
         <v>1</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>25</v>
@@ -1107,27 +1107,27 @@
         <v>1</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>25</v>
@@ -1154,27 +1154,27 @@
         <v>1</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>25</v>
@@ -1201,27 +1201,27 @@
         <v>1</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>25</v>
@@ -1248,27 +1248,27 @@
         <v>1</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>25</v>
@@ -1295,27 +1295,27 @@
         <v>1</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>25</v>
@@ -1342,27 +1342,27 @@
         <v>1</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>25</v>
@@ -1389,27 +1389,27 @@
         <v>1</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>25</v>
@@ -1436,27 +1436,27 @@
         <v>1</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>25</v>
@@ -1483,27 +1483,27 @@
         <v>1</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>25</v>
@@ -1530,27 +1530,27 @@
         <v>1</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>25</v>
@@ -1577,22 +1577,22 @@
         <v>1</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changes made: 1) PR main: - covers pure comp - outputs Z as well as rho 2) Cal main: - Automatically identifies time stamp for unique P and unique Q - Gives stats for Punique and Qunique as well as Punique and Qall - CalProcData is a struct with Fluid.T.P.Q.xxx To be done: - Cal curve with Q individual and Q all - Linear fitting - Plots each Q vs all Q together - Idea is that for individual Qs, fitting curve will be more reliable, and C estimated will be corrected by Q already. Observation: for greater Q, C was smaller, when that should not be the case, unless there is leaking!
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1019" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABBB021E-7055-4459-802D-1170FE4F6DF1}"/>
+  <xr:revisionPtr revIDLastSave="1035" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42CB1D6B-01AD-4DBE-B494-6656A1D152D8}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="1695" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25845" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="56">
   <si>
     <t>path</t>
   </si>
@@ -192,6 +192,18 @@
   </si>
   <si>
     <t>data/BP-CAL-250729/</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>ml/min</t>
+  </si>
+  <si>
+    <t>1,2,5,10</t>
+  </si>
+  <si>
+    <t>0,50,200,500,900,1500</t>
   </si>
 </sst>
 </file>
@@ -523,25 +535,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
-    <col min="3" max="6" width="7.28515625" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="6.5703125" customWidth="1"/>
-    <col min="10" max="10" width="43.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="26" style="1" customWidth="1"/>
-    <col min="14" max="14" width="18.28515625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="20.28515625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="11.7109375" customWidth="1"/>
+    <col min="3" max="4" width="7.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" customWidth="1"/>
+    <col min="11" max="11" width="43.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="26" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.28515625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="20.28515625" style="2" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -557,41 +572,44 @@
       <c r="E1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="L1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
@@ -601,20 +619,23 @@
       <c r="E2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="F2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N2" s="1"/>
       <c r="O2" s="1"/>
-    </row>
-    <row r="3" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P2" s="1"/>
+    </row>
+    <row r="3" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -627,39 +648,44 @@
       <c r="D3" s="1">
         <v>32</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3">
+      <c r="E3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3">
         <v>45867.647418981483</v>
       </c>
-      <c r="H3" s="3">
+      <c r="I3" s="3">
         <v>45867.67083333333</v>
       </c>
-      <c r="I3" s="1">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>51</v>
+      <c r="J3" s="1">
+        <v>1</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -672,39 +698,44 @@
       <c r="D4" s="1">
         <v>32</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3">
+      <c r="E4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3">
         <v>45867.576388888891</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>45867.627083333333</v>
       </c>
-      <c r="I4" s="1">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>51</v>
+      <c r="J4" s="1">
+        <v>1</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -717,39 +748,44 @@
       <c r="D5" s="1">
         <v>32</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1">
-        <v>1</v>
-      </c>
-      <c r="G5" s="3">
+      <c r="E5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3">
         <v>45867.673611111109</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>45867.716666666667</v>
       </c>
-      <c r="I5" s="1">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>51</v>
+      <c r="J5" s="1">
+        <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -765,38 +801,41 @@
       <c r="E6" s="1">
         <v>0</v>
       </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3">
+      <c r="F6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3">
         <v>45867.641504629632</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="3">
         <v>45867.651099537034</v>
       </c>
-      <c r="I6" s="1">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>51</v>
+      <c r="J6" s="1">
+        <v>1</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -812,38 +851,41 @@
       <c r="E7" s="1">
         <v>50</v>
       </c>
-      <c r="F7" s="1">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3">
+      <c r="F7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1</v>
+      </c>
+      <c r="H7" s="3">
         <v>45867.652222222219</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>45867.656122685185</v>
       </c>
-      <c r="I7" s="1">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>51</v>
+      <c r="J7" s="1">
+        <v>1</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -859,38 +901,41 @@
       <c r="E8" s="1">
         <v>200</v>
       </c>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3">
+      <c r="F8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3">
         <v>45867.65729166667</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="3">
         <v>45867.660219907404</v>
       </c>
-      <c r="I8" s="1">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>51</v>
+      <c r="J8" s="1">
+        <v>1</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -906,38 +951,41 @@
       <c r="E9" s="1">
         <v>500</v>
       </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-      <c r="G9" s="3">
+      <c r="F9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="H9" s="3">
         <v>45867.661192129628</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>45867.663587962961</v>
       </c>
-      <c r="I9" s="1">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>51</v>
+      <c r="J9" s="1">
+        <v>1</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -953,38 +1001,41 @@
       <c r="E10" s="1">
         <v>900</v>
       </c>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-      <c r="G10" s="3">
+      <c r="F10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1</v>
+      </c>
+      <c r="H10" s="3">
         <v>45867.664930555555</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>45867.667314814818</v>
       </c>
-      <c r="I10" s="1">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>51</v>
+      <c r="J10" s="1">
+        <v>1</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -1000,38 +1051,41 @@
       <c r="E11" s="1">
         <v>1500</v>
       </c>
-      <c r="F11" s="1">
-        <v>1</v>
-      </c>
-      <c r="G11" s="3">
+      <c r="F11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1</v>
+      </c>
+      <c r="H11" s="3">
         <v>45867.66846064815</v>
       </c>
-      <c r="H11" s="3">
+      <c r="I11" s="3">
         <v>45867.670763888891</v>
       </c>
-      <c r="I11" s="1">
-        <v>1</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>51</v>
+      <c r="J11" s="1">
+        <v>1</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1047,38 +1101,41 @@
       <c r="E12" s="1">
         <v>0</v>
       </c>
-      <c r="F12" s="1">
-        <v>1</v>
-      </c>
-      <c r="G12" s="3">
+      <c r="F12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1</v>
+      </c>
+      <c r="H12" s="3">
         <v>45867.58730324074</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="3">
         <v>45867.592511574076</v>
       </c>
-      <c r="I12" s="1">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>51</v>
+      <c r="J12" s="1">
+        <v>1</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -1094,38 +1151,41 @@
       <c r="E13" s="1">
         <v>50</v>
       </c>
-      <c r="F13" s="1">
-        <v>1</v>
-      </c>
-      <c r="G13" s="3">
+      <c r="F13" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1</v>
+      </c>
+      <c r="H13" s="3">
         <v>45867.595069444447</v>
       </c>
-      <c r="H13" s="3">
+      <c r="I13" s="3">
         <v>45867.603495370371</v>
       </c>
-      <c r="I13" s="1">
-        <v>1</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>51</v>
+      <c r="J13" s="1">
+        <v>1</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -1141,38 +1201,41 @@
       <c r="E14" s="1">
         <v>200</v>
       </c>
-      <c r="F14" s="1">
-        <v>1</v>
-      </c>
-      <c r="G14" s="3">
+      <c r="F14" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
+      <c r="H14" s="3">
         <v>45867.605775462966</v>
       </c>
-      <c r="H14" s="3">
+      <c r="I14" s="3">
         <v>45867.610775462963</v>
       </c>
-      <c r="I14" s="1">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>51</v>
+      <c r="J14" s="1">
+        <v>1</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>41</v>
       </c>
@@ -1188,38 +1251,41 @@
       <c r="E15" s="1">
         <v>500</v>
       </c>
-      <c r="F15" s="1">
-        <v>1</v>
-      </c>
-      <c r="G15" s="3">
+      <c r="F15" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
+      <c r="H15" s="3">
         <v>45867.613449074073</v>
       </c>
-      <c r="H15" s="3">
+      <c r="I15" s="3">
         <v>45867.615995370368</v>
       </c>
-      <c r="I15" s="1">
-        <v>1</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>51</v>
+      <c r="J15" s="1">
+        <v>1</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1235,38 +1301,41 @@
       <c r="E16" s="1">
         <v>900</v>
       </c>
-      <c r="F16" s="1">
-        <v>1</v>
-      </c>
-      <c r="G16" s="3">
+      <c r="F16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1</v>
+      </c>
+      <c r="H16" s="3">
         <v>45867.617766203701</v>
       </c>
-      <c r="H16" s="3">
+      <c r="I16" s="3">
         <v>45867.621435185189</v>
       </c>
-      <c r="I16" s="1">
-        <v>1</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>51</v>
+      <c r="J16" s="1">
+        <v>1</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -1282,38 +1351,41 @@
       <c r="E17" s="1">
         <v>1500</v>
       </c>
-      <c r="F17" s="1">
-        <v>1</v>
-      </c>
-      <c r="G17" s="3">
+      <c r="F17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1</v>
+      </c>
+      <c r="H17" s="3">
         <v>45867.623032407406</v>
       </c>
-      <c r="H17" s="3">
+      <c r="I17" s="3">
         <v>45867.627083333333</v>
       </c>
-      <c r="I17" s="1">
-        <v>1</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>51</v>
+      <c r="J17" s="1">
+        <v>1</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -1329,38 +1401,41 @@
       <c r="E18" s="1">
         <v>0</v>
       </c>
-      <c r="F18" s="1">
-        <v>1</v>
-      </c>
-      <c r="G18" s="3">
+      <c r="F18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="1">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3">
         <v>45867.683807870373</v>
       </c>
-      <c r="H18" s="3">
+      <c r="I18" s="3">
         <v>45867.688275462962</v>
       </c>
-      <c r="I18" s="1">
-        <v>1</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>51</v>
+      <c r="J18" s="1">
+        <v>1</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>45</v>
       </c>
@@ -1376,38 +1451,41 @@
       <c r="E19" s="1">
         <v>50</v>
       </c>
-      <c r="F19" s="1">
-        <v>1</v>
-      </c>
-      <c r="G19" s="3">
+      <c r="F19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1</v>
+      </c>
+      <c r="H19" s="3">
         <v>45867.695300925923</v>
       </c>
-      <c r="H19" s="3">
+      <c r="I19" s="3">
         <v>45867.697893518518</v>
       </c>
-      <c r="I19" s="1">
-        <v>1</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>51</v>
+      <c r="J19" s="1">
+        <v>1</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>46</v>
       </c>
@@ -1423,38 +1501,41 @@
       <c r="E20" s="1">
         <v>200</v>
       </c>
-      <c r="F20" s="1">
-        <v>1</v>
-      </c>
-      <c r="G20" s="3">
+      <c r="F20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="1">
+        <v>1</v>
+      </c>
+      <c r="H20" s="3">
         <v>45867.691388888888</v>
       </c>
-      <c r="H20" s="3">
+      <c r="I20" s="3">
         <v>45867.693611111114</v>
       </c>
-      <c r="I20" s="1">
-        <v>1</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>51</v>
+      <c r="J20" s="1">
+        <v>1</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -1470,38 +1551,41 @@
       <c r="E21" s="1">
         <v>500</v>
       </c>
-      <c r="F21" s="1">
-        <v>1</v>
-      </c>
-      <c r="G21" s="3">
+      <c r="F21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="1">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3">
         <v>45867.706435185188</v>
       </c>
-      <c r="H21" s="3">
+      <c r="I21" s="3">
         <v>45867.709756944445</v>
       </c>
-      <c r="I21" s="1">
-        <v>1</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>51</v>
+      <c r="J21" s="1">
+        <v>1</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -1517,38 +1601,41 @@
       <c r="E22" s="1">
         <v>900</v>
       </c>
-      <c r="F22" s="1">
-        <v>1</v>
-      </c>
-      <c r="G22" s="3">
+      <c r="F22" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="1">
+        <v>1</v>
+      </c>
+      <c r="H22" s="3">
         <v>45867.699548611112</v>
       </c>
-      <c r="H22" s="3">
+      <c r="I22" s="3">
         <v>45867.702037037037</v>
       </c>
-      <c r="I22" s="1">
-        <v>1</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>51</v>
+      <c r="J22" s="1">
+        <v>1</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -1564,300 +1651,327 @@
       <c r="E23" s="1">
         <v>1500</v>
       </c>
-      <c r="F23" s="1">
-        <v>1</v>
-      </c>
-      <c r="G23" s="3">
+      <c r="F23" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
+      </c>
+      <c r="H23" s="3">
         <v>45867.713587962964</v>
       </c>
-      <c r="H23" s="3">
+      <c r="I23" s="3">
         <v>45867.716643518521</v>
       </c>
-      <c r="I23" s="1">
-        <v>1</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>51</v>
+      <c r="J23" s="1">
+        <v>1</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-      <c r="G24" s="3"/>
+      <c r="G24" s="1"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="1"/>
-      <c r="N24" s="1"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-      <c r="G25" s="3"/>
+      <c r="G25" s="1"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="1"/>
-      <c r="N25" s="1"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="3"/>
+      <c r="G26" s="1"/>
       <c r="H26" s="3"/>
-      <c r="I26" s="1"/>
-      <c r="N26" s="1"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-      <c r="G27" s="3"/>
+      <c r="G27" s="1"/>
       <c r="H27" s="3"/>
-      <c r="I27" s="1"/>
-      <c r="N27" s="1"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="1"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q27" s="1"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="G28" s="3"/>
+      <c r="G28" s="1"/>
       <c r="H28" s="3"/>
-      <c r="I28" s="1"/>
-      <c r="N28" s="1"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q28" s="1"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
-      <c r="G29" s="3"/>
+      <c r="G29" s="1"/>
       <c r="H29" s="3"/>
-      <c r="I29" s="1"/>
-      <c r="N29" s="1"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="1"/>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q29" s="1"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-      <c r="G30" s="3"/>
+      <c r="G30" s="1"/>
       <c r="H30" s="3"/>
-      <c r="I30" s="1"/>
-      <c r="N30" s="1"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="1"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q30" s="1"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-      <c r="G31" s="3"/>
+      <c r="G31" s="1"/>
       <c r="H31" s="3"/>
-      <c r="I31" s="1"/>
-      <c r="N31" s="1"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="1"/>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q31" s="1"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
-      <c r="G32" s="3"/>
+      <c r="G32" s="1"/>
       <c r="H32" s="3"/>
-      <c r="I32" s="1"/>
-      <c r="N32" s="1"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="1"/>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
-    </row>
-    <row r="33" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q32" s="1"/>
+    </row>
+    <row r="33" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
-      <c r="G33" s="3"/>
+      <c r="G33" s="1"/>
       <c r="H33" s="3"/>
-      <c r="I33" s="1"/>
-      <c r="N33" s="1"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="1"/>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
-    </row>
-    <row r="34" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q33" s="1"/>
+    </row>
+    <row r="34" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
-      <c r="G34" s="3"/>
+      <c r="G34" s="1"/>
       <c r="H34" s="3"/>
-      <c r="I34" s="1"/>
-      <c r="N34" s="1"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
-    </row>
-    <row r="35" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q34" s="1"/>
+    </row>
+    <row r="35" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
-      <c r="G35" s="3"/>
+      <c r="G35" s="1"/>
       <c r="H35" s="3"/>
-      <c r="I35" s="1"/>
-      <c r="N35" s="1"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="1"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
-    </row>
-    <row r="36" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q35" s="1"/>
+    </row>
+    <row r="36" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
-      <c r="G36" s="3"/>
+      <c r="G36" s="1"/>
       <c r="H36" s="3"/>
-      <c r="I36" s="1"/>
-      <c r="N36" s="1"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="1"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
-    </row>
-    <row r="37" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q36" s="1"/>
+    </row>
+    <row r="37" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="3"/>
+      <c r="G37" s="1"/>
       <c r="H37" s="3"/>
-      <c r="I37" s="1"/>
-      <c r="N37" s="1"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="1"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
-    </row>
-    <row r="38" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q37" s="1"/>
+    </row>
+    <row r="38" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
-      <c r="G38" s="3"/>
+      <c r="G38" s="1"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="1"/>
-      <c r="N38" s="1"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="1"/>
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
-    </row>
-    <row r="39" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q38" s="1"/>
+    </row>
+    <row r="39" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
-      <c r="G39" s="3"/>
+      <c r="G39" s="1"/>
       <c r="H39" s="3"/>
-      <c r="I39" s="1"/>
-      <c r="N39" s="1"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="1"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
-    </row>
-    <row r="40" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q39" s="1"/>
+    </row>
+    <row r="40" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
-      <c r="G40" s="3"/>
+      <c r="G40" s="1"/>
       <c r="H40" s="3"/>
-      <c r="I40" s="1"/>
-      <c r="N40" s="1"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="1"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
-    </row>
-    <row r="41" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q40" s="1"/>
+    </row>
+    <row r="41" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
-      <c r="G41" s="3"/>
+      <c r="G41" s="1"/>
       <c r="H41" s="3"/>
-      <c r="I41" s="1"/>
-      <c r="N41" s="1"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
-    </row>
-    <row r="42" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q41" s="1"/>
+    </row>
+    <row r="42" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
-      <c r="G42" s="3"/>
+      <c r="G42" s="1"/>
       <c r="H42" s="3"/>
-      <c r="I42" s="1"/>
-      <c r="N42" s="1"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="1"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
-    </row>
-    <row r="43" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q42" s="1"/>
+    </row>
+    <row r="43" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
-      <c r="G43" s="3"/>
+      <c r="G43" s="1"/>
       <c r="H43" s="3"/>
-      <c r="I43" s="1"/>
-      <c r="N43" s="1"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="1"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
-    </row>
-    <row r="44" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q43" s="1"/>
+    </row>
+    <row r="44" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
-      <c r="G44" s="3"/>
+      <c r="G44" s="1"/>
       <c r="H44" s="3"/>
-      <c r="I44" s="1"/>
-      <c r="N44" s="1"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="1"/>
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
-    </row>
-    <row r="45" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q44" s="1"/>
+    </row>
+    <row r="45" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-      <c r="G45" s="3"/>
+      <c r="G45" s="1"/>
       <c r="H45" s="3"/>
-      <c r="I45" s="1"/>
-      <c r="N45" s="1"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="1"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
-    </row>
-    <row r="46" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q45" s="1"/>
+    </row>
+    <row r="46" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
-      <c r="G46" s="3"/>
+      <c r="G46" s="1"/>
       <c r="H46" s="3"/>
-      <c r="I46" s="1"/>
-      <c r="N46" s="1"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="1"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
-    </row>
-    <row r="47" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="Q46" s="1"/>
+    </row>
+    <row r="47" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
-      <c r="G47" s="3"/>
+      <c r="G47" s="1"/>
       <c r="H47" s="3"/>
-      <c r="I47" s="1"/>
-      <c r="N47" s="1"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="1"/>
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
+      <c r="Q47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
time adjusted in input of CO2 such that itt captures only when temperature started to stabilize
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1035" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42CB1D6B-01AD-4DBE-B494-6656A1D152D8}"/>
+  <xr:revisionPtr revIDLastSave="1036" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE4BAE8A-1050-4C0F-AFB3-E85B8EDED879}"/>
   <bookViews>
-    <workbookView xWindow="-25845" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26010" yWindow="1740" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="3">
-        <v>45867.673611111109</v>
+        <v>45867.682719907411</v>
       </c>
       <c r="I5" s="3">
         <v>45867.716666666667</v>

</xml_diff>

<commit_message>
Import options for pump dat was changed to allow to know the number of the pump for working, confining and cushion, as for different experiments, the number of the pump may have changed, for example pump 3 previously used for confining, it was later used for working, etc. This also allows to have P toal and Q total, wothout adding up the two probable pumps working
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1037" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE47F218-14A7-4256-90A0-8718D225DCDE}"/>
+  <xr:revisionPtr revIDLastSave="1049" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7D9A2B6-634D-4229-9E11-659C87FD121A}"/>
   <bookViews>
-    <workbookView xWindow="-26775" yWindow="2745" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23850" yWindow="2970" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
   <si>
     <t>path</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>0,50,200,500,900,1500</t>
+  </si>
+  <si>
+    <t>workingPump</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.44140625" customWidth="1"/>
@@ -490,19 +493,20 @@
     <col min="5" max="5" width="20.6640625" customWidth="1"/>
     <col min="6" max="6" width="11.44140625" customWidth="1"/>
     <col min="7" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="8" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" customWidth="1"/>
-    <col min="11" max="11" width="43.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.33203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="26" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.33203125" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.33203125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="11.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" customWidth="1"/>
+    <col min="11" max="11" width="6.5546875" customWidth="1"/>
+    <col min="12" max="12" width="43.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.33203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="26" style="1" customWidth="1"/>
+    <col min="16" max="16" width="18.33203125" style="2" customWidth="1"/>
+    <col min="17" max="17" width="20.33203125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -525,37 +529,40 @@
         <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
@@ -569,19 +576,20 @@
         <v>35</v>
       </c>
       <c r="G2" s="1"/>
-      <c r="H2" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="1"/>
       <c r="P2" s="1"/>
-    </row>
-    <row r="3" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -603,35 +611,38 @@
       <c r="G3" s="1">
         <v>1</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3">
         <v>45867.647418981483</v>
       </c>
-      <c r="I3" s="3">
+      <c r="J3" s="3">
         <v>45867.67083333333</v>
       </c>
-      <c r="J3" s="1">
+      <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -653,35 +664,38 @@
       <c r="G4" s="1">
         <v>1</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3">
         <v>45867.576388888891</v>
       </c>
-      <c r="I4" s="3">
+      <c r="J4" s="3">
         <v>45867.627083333333</v>
       </c>
-      <c r="J4" s="1">
+      <c r="K4" s="1">
         <v>1</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -703,501 +717,546 @@
       <c r="G5" s="1">
         <v>1</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="1">
+        <v>2</v>
+      </c>
+      <c r="I5" s="3">
         <v>45867.682719907411</v>
       </c>
-      <c r="I5" s="3">
+      <c r="J5" s="3">
         <v>45867.716666666667</v>
       </c>
-      <c r="J5" s="1">
+      <c r="K5" s="1">
         <v>1</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="R5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
-      <c r="H6" s="3"/>
+      <c r="H6" s="1"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="1"/>
-      <c r="Q6" s="1"/>
-    </row>
-    <row r="7" spans="1:17" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J6" s="3"/>
+      <c r="K6" s="1"/>
+      <c r="R6" s="1"/>
+    </row>
+    <row r="7" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="H7" s="3"/>
+      <c r="H7" s="1"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="1"/>
-      <c r="Q7" s="1"/>
-    </row>
-    <row r="8" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J7" s="3"/>
+      <c r="K7" s="1"/>
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
-      <c r="H8" s="3"/>
+      <c r="H8" s="1"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="1"/>
-      <c r="Q8" s="1"/>
-    </row>
-    <row r="9" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J8" s="3"/>
+      <c r="K8" s="1"/>
+      <c r="R8" s="1"/>
+    </row>
+    <row r="9" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="3"/>
+      <c r="H9" s="1"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="1"/>
-      <c r="Q9" s="1"/>
-    </row>
-    <row r="10" spans="1:17" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J9" s="3"/>
+      <c r="K9" s="1"/>
+      <c r="R9" s="1"/>
+    </row>
+    <row r="10" spans="1:18" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="1"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="1"/>
-      <c r="Q10" s="1"/>
-    </row>
-    <row r="11" spans="1:17" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J10" s="3"/>
+      <c r="K10" s="1"/>
+      <c r="R10" s="1"/>
+    </row>
+    <row r="11" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="3"/>
+      <c r="H11" s="1"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="1"/>
-      <c r="Q11" s="1"/>
-    </row>
-    <row r="12" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J11" s="3"/>
+      <c r="K11" s="1"/>
+      <c r="R11" s="1"/>
+    </row>
+    <row r="12" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="3"/>
+      <c r="H12" s="1"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="1"/>
-      <c r="Q12" s="1"/>
-    </row>
-    <row r="13" spans="1:17" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J12" s="3"/>
+      <c r="K12" s="1"/>
+      <c r="R12" s="1"/>
+    </row>
+    <row r="13" spans="1:18" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="3"/>
+      <c r="H13" s="1"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="1"/>
-      <c r="Q13" s="1"/>
-    </row>
-    <row r="14" spans="1:17" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J13" s="3"/>
+      <c r="K13" s="1"/>
+      <c r="R13" s="1"/>
+    </row>
+    <row r="14" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="3"/>
+      <c r="H14" s="1"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="1"/>
-      <c r="Q14" s="1"/>
-    </row>
-    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J14" s="3"/>
+      <c r="K14" s="1"/>
+      <c r="R14" s="1"/>
+    </row>
+    <row r="15" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
-      <c r="H15" s="3"/>
+      <c r="H15" s="1"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="1"/>
-      <c r="Q15" s="1"/>
-    </row>
-    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J15" s="3"/>
+      <c r="K15" s="1"/>
+      <c r="R15" s="1"/>
+    </row>
+    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
-      <c r="H16" s="3"/>
+      <c r="H16" s="1"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="1"/>
-      <c r="Q16" s="1"/>
-    </row>
-    <row r="17" spans="4:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J16" s="3"/>
+      <c r="K16" s="1"/>
+      <c r="R16" s="1"/>
+    </row>
+    <row r="17" spans="4:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="3"/>
+      <c r="H17" s="1"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="1"/>
-      <c r="Q17" s="1"/>
-    </row>
-    <row r="18" spans="4:17" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J17" s="3"/>
+      <c r="K17" s="1"/>
+      <c r="R17" s="1"/>
+    </row>
+    <row r="18" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
-      <c r="H18" s="3"/>
+      <c r="H18" s="1"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="1"/>
-      <c r="Q18" s="1"/>
-    </row>
-    <row r="19" spans="4:17" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J18" s="3"/>
+      <c r="K18" s="1"/>
+      <c r="R18" s="1"/>
+    </row>
+    <row r="19" spans="4:18" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
-      <c r="H19" s="3"/>
+      <c r="H19" s="1"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="1"/>
-      <c r="Q19" s="1"/>
-    </row>
-    <row r="20" spans="4:17" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J19" s="3"/>
+      <c r="K19" s="1"/>
+      <c r="R19" s="1"/>
+    </row>
+    <row r="20" spans="4:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
-      <c r="H20" s="3"/>
+      <c r="H20" s="1"/>
       <c r="I20" s="3"/>
-      <c r="J20" s="1"/>
-      <c r="Q20" s="1"/>
-    </row>
-    <row r="21" spans="4:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J20" s="3"/>
+      <c r="K20" s="1"/>
+      <c r="R20" s="1"/>
+    </row>
+    <row r="21" spans="4:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
-      <c r="H21" s="3"/>
+      <c r="H21" s="1"/>
       <c r="I21" s="3"/>
-      <c r="J21" s="1"/>
-      <c r="Q21" s="1"/>
-    </row>
-    <row r="22" spans="4:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J21" s="3"/>
+      <c r="K21" s="1"/>
+      <c r="R21" s="1"/>
+    </row>
+    <row r="22" spans="4:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
-      <c r="H22" s="3"/>
+      <c r="H22" s="1"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="1"/>
-      <c r="Q22" s="1"/>
-    </row>
-    <row r="23" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J22" s="3"/>
+      <c r="K22" s="1"/>
+      <c r="R22" s="1"/>
+    </row>
+    <row r="23" spans="4:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
-      <c r="H23" s="3"/>
+      <c r="H23" s="1"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="1"/>
-      <c r="Q23" s="1"/>
-    </row>
-    <row r="24" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="J23" s="3"/>
+      <c r="K23" s="1"/>
+      <c r="R23" s="1"/>
+    </row>
+    <row r="24" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
-      <c r="H24" s="3"/>
+      <c r="H24" s="1"/>
       <c r="I24" s="3"/>
-      <c r="J24" s="1"/>
-      <c r="O24" s="1"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="1"/>
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
-    </row>
-    <row r="25" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R24" s="1"/>
+    </row>
+    <row r="25" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
-      <c r="H25" s="3"/>
+      <c r="H25" s="1"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="1"/>
-      <c r="O25" s="1"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
-    </row>
-    <row r="26" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R25" s="1"/>
+    </row>
+    <row r="26" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="3"/>
+      <c r="H26" s="1"/>
       <c r="I26" s="3"/>
-      <c r="J26" s="1"/>
-      <c r="O26" s="1"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
-    </row>
-    <row r="27" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R26" s="1"/>
+    </row>
+    <row r="27" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
-      <c r="H27" s="3"/>
+      <c r="H27" s="1"/>
       <c r="I27" s="3"/>
-      <c r="J27" s="1"/>
-      <c r="O27" s="1"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="1"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
-    </row>
-    <row r="28" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R27" s="1"/>
+    </row>
+    <row r="28" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
-      <c r="H28" s="3"/>
+      <c r="H28" s="1"/>
       <c r="I28" s="3"/>
-      <c r="J28" s="1"/>
-      <c r="O28" s="1"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="1"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
-    </row>
-    <row r="29" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R28" s="1"/>
+    </row>
+    <row r="29" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-      <c r="H29" s="3"/>
+      <c r="H29" s="1"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="1"/>
-      <c r="O29" s="1"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
-    </row>
-    <row r="30" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R29" s="1"/>
+    </row>
+    <row r="30" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
-      <c r="H30" s="3"/>
+      <c r="H30" s="1"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="1"/>
-      <c r="O30" s="1"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
-    </row>
-    <row r="31" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R30" s="1"/>
+    </row>
+    <row r="31" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-      <c r="H31" s="3"/>
+      <c r="H31" s="1"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="1"/>
-      <c r="O31" s="1"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="1"/>
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
-    </row>
-    <row r="32" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R31" s="1"/>
+    </row>
+    <row r="32" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
-      <c r="H32" s="3"/>
+      <c r="H32" s="1"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="1"/>
-      <c r="O32" s="1"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="1"/>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
-    </row>
-    <row r="33" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R32" s="1"/>
+    </row>
+    <row r="33" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
-      <c r="H33" s="3"/>
+      <c r="H33" s="1"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="1"/>
-      <c r="O33" s="1"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="1"/>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
-    </row>
-    <row r="34" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R33" s="1"/>
+    </row>
+    <row r="34" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
-      <c r="H34" s="3"/>
+      <c r="H34" s="1"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="1"/>
-      <c r="O34" s="1"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="1"/>
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
-    </row>
-    <row r="35" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R34" s="1"/>
+    </row>
+    <row r="35" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
-      <c r="H35" s="3"/>
+      <c r="H35" s="1"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="1"/>
-      <c r="O35" s="1"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
-    </row>
-    <row r="36" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R35" s="1"/>
+    </row>
+    <row r="36" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
-      <c r="H36" s="3"/>
+      <c r="H36" s="1"/>
       <c r="I36" s="3"/>
-      <c r="J36" s="1"/>
-      <c r="O36" s="1"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="1"/>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
-    </row>
-    <row r="37" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R36" s="1"/>
+    </row>
+    <row r="37" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
-      <c r="H37" s="3"/>
+      <c r="H37" s="1"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="1"/>
-      <c r="O37" s="1"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="1"/>
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
-    </row>
-    <row r="38" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R37" s="1"/>
+    </row>
+    <row r="38" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
-      <c r="H38" s="3"/>
+      <c r="H38" s="1"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="1"/>
-      <c r="O38" s="1"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="1"/>
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
-    </row>
-    <row r="39" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R38" s="1"/>
+    </row>
+    <row r="39" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
-      <c r="H39" s="3"/>
+      <c r="H39" s="1"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="1"/>
-      <c r="O39" s="1"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
-    </row>
-    <row r="40" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R39" s="1"/>
+    </row>
+    <row r="40" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
-      <c r="H40" s="3"/>
+      <c r="H40" s="1"/>
       <c r="I40" s="3"/>
-      <c r="J40" s="1"/>
-      <c r="O40" s="1"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
-    </row>
-    <row r="41" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R40" s="1"/>
+    </row>
+    <row r="41" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
-      <c r="H41" s="3"/>
+      <c r="H41" s="1"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="1"/>
-      <c r="O41" s="1"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="1"/>
       <c r="P41" s="1"/>
       <c r="Q41" s="1"/>
-    </row>
-    <row r="42" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R41" s="1"/>
+    </row>
+    <row r="42" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
-      <c r="H42" s="3"/>
+      <c r="H42" s="1"/>
       <c r="I42" s="3"/>
-      <c r="J42" s="1"/>
-      <c r="O42" s="1"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
-    </row>
-    <row r="43" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R42" s="1"/>
+    </row>
+    <row r="43" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
-      <c r="H43" s="3"/>
+      <c r="H43" s="1"/>
       <c r="I43" s="3"/>
-      <c r="J43" s="1"/>
-      <c r="O43" s="1"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
-    </row>
-    <row r="44" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R43" s="1"/>
+    </row>
+    <row r="44" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
-      <c r="H44" s="3"/>
+      <c r="H44" s="1"/>
       <c r="I44" s="3"/>
-      <c r="J44" s="1"/>
-      <c r="O44" s="1"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="1"/>
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
-    </row>
-    <row r="45" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R44" s="1"/>
+    </row>
+    <row r="45" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
-      <c r="H45" s="3"/>
+      <c r="H45" s="1"/>
       <c r="I45" s="3"/>
-      <c r="J45" s="1"/>
-      <c r="O45" s="1"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
-    </row>
-    <row r="46" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R45" s="1"/>
+    </row>
+    <row r="46" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
-      <c r="H46" s="3"/>
+      <c r="H46" s="1"/>
       <c r="I46" s="3"/>
-      <c r="J46" s="1"/>
-      <c r="O46" s="1"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
-    </row>
-    <row r="47" spans="4:17" x14ac:dyDescent="0.3">
+      <c r="R46" s="1"/>
+    </row>
+    <row r="47" spans="4:18" x14ac:dyDescent="0.3">
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
-      <c r="H47" s="3"/>
+      <c r="H47" s="1"/>
       <c r="I47" s="3"/>
-      <c r="J47" s="1"/>
-      <c r="O47" s="1"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="1"/>
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
+      <c r="R47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
main Cal with input file changed to add Fluid2 to use same function for main_val
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1049" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7D9A2B6-634D-4229-9E11-659C87FD121A}"/>
+  <xr:revisionPtr revIDLastSave="1051" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B776A18-96A0-4377-B840-542D96AFF726}"/>
   <bookViews>
-    <workbookView xWindow="-23850" yWindow="2970" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>path</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>workingPump</t>
+  </si>
+  <si>
+    <t>Fluid2</t>
   </si>
 </sst>
 </file>
@@ -484,29 +487,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S47"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" style="4" customWidth="1"/>
-    <col min="3" max="4" width="7.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" customWidth="1"/>
-    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5546875" customWidth="1"/>
-    <col min="11" max="11" width="6.5546875" customWidth="1"/>
-    <col min="12" max="12" width="43.109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.33203125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="26" style="1" customWidth="1"/>
-    <col min="16" max="16" width="18.33203125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="20.33203125" style="2" customWidth="1"/>
-    <col min="18" max="18" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
+    <col min="3" max="5" width="7.28515625" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" customWidth="1"/>
+    <col min="13" max="13" width="43.140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.28515625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="26" style="1" customWidth="1"/>
+    <col min="17" max="17" width="18.28515625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="20.28515625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -516,80 +519,83 @@
       <c r="C1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
-    </row>
-    <row r="3" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -599,50 +605,50 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>32</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
       </c>
       <c r="H3" s="1">
         <v>1</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="3">
         <v>45867.647418981483</v>
       </c>
-      <c r="J3" s="3">
+      <c r="K3" s="3">
         <v>45867.67083333333</v>
       </c>
-      <c r="K3" s="1">
+      <c r="L3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -652,50 +658,50 @@
       <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>32</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="G4" s="1">
-        <v>1</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="1">
+        <v>1</v>
+      </c>
+      <c r="J4" s="3">
         <v>45867.576388888891</v>
       </c>
-      <c r="J4" s="3">
+      <c r="K4" s="3">
         <v>45867.627083333333</v>
       </c>
-      <c r="K4" s="1">
+      <c r="L4" s="1">
         <v>1</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -705,558 +711,558 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>32</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>1</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>2</v>
       </c>
-      <c r="I5" s="3">
+      <c r="J5" s="3">
         <v>45867.682719907411</v>
       </c>
-      <c r="J5" s="3">
+      <c r="K5" s="3">
         <v>45867.716666666667</v>
       </c>
-      <c r="K5" s="1">
+      <c r="L5" s="1">
         <v>1</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D6" s="1"/>
+    <row r="6" spans="1:19" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="3"/>
+      <c r="I6" s="1"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="1"/>
-      <c r="R6" s="1"/>
-    </row>
-    <row r="7" spans="1:18" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D7" s="1"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="1"/>
+      <c r="S6" s="1"/>
+    </row>
+    <row r="7" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="3"/>
+      <c r="I7" s="1"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="1"/>
-      <c r="R7" s="1"/>
-    </row>
-    <row r="8" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D8" s="1"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="1"/>
+      <c r="S7" s="1"/>
+    </row>
+    <row r="8" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="3"/>
+      <c r="I8" s="1"/>
       <c r="J8" s="3"/>
-      <c r="K8" s="1"/>
-      <c r="R8" s="1"/>
-    </row>
-    <row r="9" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="1"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="1"/>
+      <c r="S8" s="1"/>
+    </row>
+    <row r="9" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="I9" s="3"/>
+      <c r="I9" s="1"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="1"/>
-      <c r="R9" s="1"/>
-    </row>
-    <row r="10" spans="1:18" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="1"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="1"/>
+      <c r="S9" s="1"/>
+    </row>
+    <row r="10" spans="1:19" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="3"/>
+      <c r="I10" s="1"/>
       <c r="J10" s="3"/>
-      <c r="K10" s="1"/>
-      <c r="R10" s="1"/>
-    </row>
-    <row r="11" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D11" s="1"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="1"/>
+      <c r="S10" s="1"/>
+    </row>
+    <row r="11" spans="1:19" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="3"/>
+      <c r="I11" s="1"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="1"/>
-      <c r="R11" s="1"/>
-    </row>
-    <row r="12" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D12" s="1"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="1"/>
+      <c r="S11" s="1"/>
+    </row>
+    <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
-      <c r="I12" s="3"/>
+      <c r="I12" s="1"/>
       <c r="J12" s="3"/>
-      <c r="K12" s="1"/>
-      <c r="R12" s="1"/>
-    </row>
-    <row r="13" spans="1:18" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D13" s="1"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="1"/>
+      <c r="S12" s="1"/>
+    </row>
+    <row r="13" spans="1:19" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
-      <c r="I13" s="3"/>
+      <c r="I13" s="1"/>
       <c r="J13" s="3"/>
-      <c r="K13" s="1"/>
-      <c r="R13" s="1"/>
-    </row>
-    <row r="14" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D14" s="1"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="1"/>
+      <c r="S13" s="1"/>
+    </row>
+    <row r="14" spans="1:19" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-      <c r="I14" s="3"/>
+      <c r="I14" s="1"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="1"/>
-      <c r="R14" s="1"/>
-    </row>
-    <row r="15" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="1"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="1"/>
+      <c r="S14" s="1"/>
+    </row>
+    <row r="15" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
-      <c r="I15" s="3"/>
+      <c r="I15" s="1"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="1"/>
-      <c r="R15" s="1"/>
-    </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D16" s="1"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="1"/>
+      <c r="S15" s="1"/>
+    </row>
+    <row r="16" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
-      <c r="I16" s="3"/>
+      <c r="I16" s="1"/>
       <c r="J16" s="3"/>
-      <c r="K16" s="1"/>
-      <c r="R16" s="1"/>
-    </row>
-    <row r="17" spans="4:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="1"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="1"/>
+      <c r="S16" s="1"/>
+    </row>
+    <row r="17" spans="5:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="3"/>
+      <c r="I17" s="1"/>
       <c r="J17" s="3"/>
-      <c r="K17" s="1"/>
-      <c r="R17" s="1"/>
-    </row>
-    <row r="18" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="1"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="1"/>
+      <c r="S17" s="1"/>
+    </row>
+    <row r="18" spans="5:19" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="3"/>
+      <c r="I18" s="1"/>
       <c r="J18" s="3"/>
-      <c r="K18" s="1"/>
-      <c r="R18" s="1"/>
-    </row>
-    <row r="19" spans="4:18" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="1"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="1"/>
+      <c r="S18" s="1"/>
+    </row>
+    <row r="19" spans="5:19" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
-      <c r="I19" s="3"/>
+      <c r="I19" s="1"/>
       <c r="J19" s="3"/>
-      <c r="K19" s="1"/>
-      <c r="R19" s="1"/>
-    </row>
-    <row r="20" spans="4:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D20" s="1"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="1"/>
+      <c r="S19" s="1"/>
+    </row>
+    <row r="20" spans="5:19" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
-      <c r="I20" s="3"/>
+      <c r="I20" s="1"/>
       <c r="J20" s="3"/>
-      <c r="K20" s="1"/>
-      <c r="R20" s="1"/>
-    </row>
-    <row r="21" spans="4:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D21" s="1"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="1"/>
+      <c r="S20" s="1"/>
+    </row>
+    <row r="21" spans="5:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
-      <c r="I21" s="3"/>
+      <c r="I21" s="1"/>
       <c r="J21" s="3"/>
-      <c r="K21" s="1"/>
-      <c r="R21" s="1"/>
-    </row>
-    <row r="22" spans="4:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D22" s="1"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="1"/>
+      <c r="S21" s="1"/>
+    </row>
+    <row r="22" spans="5:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="3"/>
+      <c r="I22" s="1"/>
       <c r="J22" s="3"/>
-      <c r="K22" s="1"/>
-      <c r="R22" s="1"/>
-    </row>
-    <row r="23" spans="4:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D23" s="1"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="1"/>
+      <c r="S22" s="1"/>
+    </row>
+    <row r="23" spans="5:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="3"/>
+      <c r="I23" s="1"/>
       <c r="J23" s="3"/>
-      <c r="K23" s="1"/>
-      <c r="R23" s="1"/>
-    </row>
-    <row r="24" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D24" s="1"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="1"/>
+      <c r="S23" s="1"/>
+    </row>
+    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="3"/>
+      <c r="I24" s="1"/>
       <c r="J24" s="3"/>
-      <c r="K24" s="1"/>
-      <c r="P24" s="1"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="1"/>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
-    </row>
-    <row r="25" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D25" s="1"/>
+      <c r="S24" s="1"/>
+    </row>
+    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
-      <c r="I25" s="3"/>
+      <c r="I25" s="1"/>
       <c r="J25" s="3"/>
-      <c r="K25" s="1"/>
-      <c r="P25" s="1"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="1"/>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
-    </row>
-    <row r="26" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D26" s="1"/>
+      <c r="S25" s="1"/>
+    </row>
+    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="3"/>
+      <c r="I26" s="1"/>
       <c r="J26" s="3"/>
-      <c r="K26" s="1"/>
-      <c r="P26" s="1"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="1"/>
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
-    </row>
-    <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="1"/>
+      <c r="S26" s="1"/>
+    </row>
+    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="3"/>
+      <c r="I27" s="1"/>
       <c r="J27" s="3"/>
-      <c r="K27" s="1"/>
-      <c r="P27" s="1"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="1"/>
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
-    </row>
-    <row r="28" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D28" s="1"/>
+      <c r="S27" s="1"/>
+    </row>
+    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="3"/>
+      <c r="I28" s="1"/>
       <c r="J28" s="3"/>
-      <c r="K28" s="1"/>
-      <c r="P28" s="1"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="1"/>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
-    </row>
-    <row r="29" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D29" s="1"/>
+      <c r="S28" s="1"/>
+    </row>
+    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="3"/>
+      <c r="I29" s="1"/>
       <c r="J29" s="3"/>
-      <c r="K29" s="1"/>
-      <c r="P29" s="1"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="1"/>
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
-    </row>
-    <row r="30" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D30" s="1"/>
+      <c r="S29" s="1"/>
+    </row>
+    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
-      <c r="I30" s="3"/>
+      <c r="I30" s="1"/>
       <c r="J30" s="3"/>
-      <c r="K30" s="1"/>
-      <c r="P30" s="1"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="1"/>
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
-    </row>
-    <row r="31" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D31" s="1"/>
+      <c r="S30" s="1"/>
+    </row>
+    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
-      <c r="I31" s="3"/>
+      <c r="I31" s="1"/>
       <c r="J31" s="3"/>
-      <c r="K31" s="1"/>
-      <c r="P31" s="1"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="1"/>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
-    </row>
-    <row r="32" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D32" s="1"/>
+      <c r="S31" s="1"/>
+    </row>
+    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="3"/>
+      <c r="I32" s="1"/>
       <c r="J32" s="3"/>
-      <c r="K32" s="1"/>
-      <c r="P32" s="1"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="1"/>
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
-    </row>
-    <row r="33" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D33" s="1"/>
+      <c r="S32" s="1"/>
+    </row>
+    <row r="33" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
-      <c r="I33" s="3"/>
+      <c r="I33" s="1"/>
       <c r="J33" s="3"/>
-      <c r="K33" s="1"/>
-      <c r="P33" s="1"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="1"/>
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
-    </row>
-    <row r="34" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D34" s="1"/>
+      <c r="S33" s="1"/>
+    </row>
+    <row r="34" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
-      <c r="I34" s="3"/>
+      <c r="I34" s="1"/>
       <c r="J34" s="3"/>
-      <c r="K34" s="1"/>
-      <c r="P34" s="1"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="1"/>
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
-    </row>
-    <row r="35" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D35" s="1"/>
+      <c r="S34" s="1"/>
+    </row>
+    <row r="35" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
-      <c r="I35" s="3"/>
+      <c r="I35" s="1"/>
       <c r="J35" s="3"/>
-      <c r="K35" s="1"/>
-      <c r="P35" s="1"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="1"/>
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
-    </row>
-    <row r="36" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D36" s="1"/>
+      <c r="S35" s="1"/>
+    </row>
+    <row r="36" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
-      <c r="I36" s="3"/>
+      <c r="I36" s="1"/>
       <c r="J36" s="3"/>
-      <c r="K36" s="1"/>
-      <c r="P36" s="1"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="1"/>
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
-    </row>
-    <row r="37" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D37" s="1"/>
+      <c r="S36" s="1"/>
+    </row>
+    <row r="37" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
-      <c r="I37" s="3"/>
+      <c r="I37" s="1"/>
       <c r="J37" s="3"/>
-      <c r="K37" s="1"/>
-      <c r="P37" s="1"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="1"/>
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
-    </row>
-    <row r="38" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D38" s="1"/>
+      <c r="S37" s="1"/>
+    </row>
+    <row r="38" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
-      <c r="I38" s="3"/>
+      <c r="I38" s="1"/>
       <c r="J38" s="3"/>
-      <c r="K38" s="1"/>
-      <c r="P38" s="1"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="1"/>
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
-    </row>
-    <row r="39" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D39" s="1"/>
+      <c r="S38" s="1"/>
+    </row>
+    <row r="39" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
-      <c r="I39" s="3"/>
+      <c r="I39" s="1"/>
       <c r="J39" s="3"/>
-      <c r="K39" s="1"/>
-      <c r="P39" s="1"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="1"/>
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
-    </row>
-    <row r="40" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D40" s="1"/>
+      <c r="S39" s="1"/>
+    </row>
+    <row r="40" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
-      <c r="I40" s="3"/>
+      <c r="I40" s="1"/>
       <c r="J40" s="3"/>
-      <c r="K40" s="1"/>
-      <c r="P40" s="1"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="1"/>
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
-    </row>
-    <row r="41" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D41" s="1"/>
+      <c r="S40" s="1"/>
+    </row>
+    <row r="41" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
-      <c r="I41" s="3"/>
+      <c r="I41" s="1"/>
       <c r="J41" s="3"/>
-      <c r="K41" s="1"/>
-      <c r="P41" s="1"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="1"/>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
-    </row>
-    <row r="42" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D42" s="1"/>
+      <c r="S41" s="1"/>
+    </row>
+    <row r="42" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
-      <c r="I42" s="3"/>
+      <c r="I42" s="1"/>
       <c r="J42" s="3"/>
-      <c r="K42" s="1"/>
-      <c r="P42" s="1"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="1"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
-    </row>
-    <row r="43" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D43" s="1"/>
+      <c r="S42" s="1"/>
+    </row>
+    <row r="43" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
-      <c r="I43" s="3"/>
+      <c r="I43" s="1"/>
       <c r="J43" s="3"/>
-      <c r="K43" s="1"/>
-      <c r="P43" s="1"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="1"/>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
-    </row>
-    <row r="44" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D44" s="1"/>
+      <c r="S43" s="1"/>
+    </row>
+    <row r="44" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
-      <c r="I44" s="3"/>
+      <c r="I44" s="1"/>
       <c r="J44" s="3"/>
-      <c r="K44" s="1"/>
-      <c r="P44" s="1"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="1"/>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
-    </row>
-    <row r="45" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D45" s="1"/>
+      <c r="S44" s="1"/>
+    </row>
+    <row r="45" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
-      <c r="I45" s="3"/>
+      <c r="I45" s="1"/>
       <c r="J45" s="3"/>
-      <c r="K45" s="1"/>
-      <c r="P45" s="1"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="1"/>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
-    </row>
-    <row r="46" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D46" s="1"/>
+      <c r="S45" s="1"/>
+    </row>
+    <row r="46" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
-      <c r="I46" s="3"/>
+      <c r="I46" s="1"/>
       <c r="J46" s="3"/>
-      <c r="K46" s="1"/>
-      <c r="P46" s="1"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="1"/>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
-    </row>
-    <row r="47" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D47" s="1"/>
+      <c r="S46" s="1"/>
+    </row>
+    <row r="47" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
-      <c r="I47" s="3"/>
+      <c r="I47" s="1"/>
       <c r="J47" s="3"/>
-      <c r="K47" s="1"/>
-      <c r="P47" s="1"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="1"/>
       <c r="Q47" s="1"/>
       <c r="R47" s="1"/>
+      <c r="S47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
main cal changes after adding X1 ol fraction for input import file function
</commit_message>
<xml_diff>
--- a/input/input_cal_exp.xlsx
+++ b/input/input_cal_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1051" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B776A18-96A0-4377-B840-542D96AFF726}"/>
+  <xr:revisionPtr revIDLastSave="1060" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2C8DEC8-1AE8-4871-A62E-ADDC1D7A7FFA}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="42">
   <si>
     <t>path</t>
   </si>
@@ -156,6 +156,12 @@
   </si>
   <si>
     <t>Fluid2</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>mol fraction</t>
   </si>
 </sst>
 </file>
@@ -487,29 +493,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
     <col min="3" max="5" width="7.28515625" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" customWidth="1"/>
-    <col min="8" max="8" width="7.28515625" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" customWidth="1"/>
-    <col min="13" max="13" width="43.140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="26" style="1" customWidth="1"/>
-    <col min="17" max="17" width="18.28515625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="20.28515625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="7.28515625" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="6.5703125" customWidth="1"/>
+    <col min="14" max="14" width="43.140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.28515625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="26" style="1" customWidth="1"/>
+    <col min="18" max="18" width="18.28515625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="20.28515625" style="2" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -529,46 +536,49 @@
         <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
@@ -579,23 +589,26 @@
         <v>16</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="J2" s="1"/>
       <c r="K2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
-    </row>
-    <row r="3" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:20" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -611,44 +624,47 @@
       <c r="F3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1</v>
       </c>
       <c r="I3" s="1">
         <v>1</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="1">
+        <v>1</v>
+      </c>
+      <c r="K3" s="3">
         <v>45867.647418981483</v>
       </c>
-      <c r="K3" s="3">
+      <c r="L3" s="3">
         <v>45867.67083333333</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="1">
         <v>1</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="S3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="T3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -664,44 +680,47 @@
       <c r="F4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1</v>
       </c>
       <c r="I4" s="1">
         <v>1</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="1">
+        <v>1</v>
+      </c>
+      <c r="K4" s="3">
         <v>45867.576388888891</v>
       </c>
-      <c r="K4" s="3">
+      <c r="L4" s="3">
         <v>45867.627083333333</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
         <v>1</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -717,552 +736,597 @@
       <c r="F5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>1</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>2</v>
       </c>
-      <c r="J5" s="3">
+      <c r="K5" s="3">
         <v>45867.682719907411</v>
       </c>
-      <c r="K5" s="3">
+      <c r="L5" s="3">
         <v>45867.716666666667</v>
       </c>
-      <c r="L5" s="1">
+      <c r="M5" s="1">
         <v>1</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="S5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="S5" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="3"/>
+      <c r="J6" s="1"/>
       <c r="K6" s="3"/>
-      <c r="L6" s="1"/>
-      <c r="S6" s="1"/>
-    </row>
-    <row r="7" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="3"/>
+      <c r="M6" s="1"/>
+      <c r="T6" s="1"/>
+    </row>
+    <row r="7" spans="1:20" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="3"/>
+      <c r="J7" s="1"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="1"/>
-      <c r="S7" s="1"/>
-    </row>
-    <row r="8" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L7" s="3"/>
+      <c r="M7" s="1"/>
+      <c r="T7" s="1"/>
+    </row>
+    <row r="8" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="3"/>
+      <c r="J8" s="1"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="1"/>
-      <c r="S8" s="1"/>
-    </row>
-    <row r="9" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L8" s="3"/>
+      <c r="M8" s="1"/>
+      <c r="T8" s="1"/>
+    </row>
+    <row r="9" spans="1:20" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="3"/>
+      <c r="J9" s="1"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="1"/>
-      <c r="S9" s="1"/>
-    </row>
-    <row r="10" spans="1:19" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L9" s="3"/>
+      <c r="M9" s="1"/>
+      <c r="T9" s="1"/>
+    </row>
+    <row r="10" spans="1:20" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="3"/>
+      <c r="J10" s="1"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="1"/>
-      <c r="S10" s="1"/>
-    </row>
-    <row r="11" spans="1:19" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L10" s="3"/>
+      <c r="M10" s="1"/>
+      <c r="T10" s="1"/>
+    </row>
+    <row r="11" spans="1:20" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="3"/>
+      <c r="J11" s="1"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="1"/>
-      <c r="S11" s="1"/>
-    </row>
-    <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L11" s="3"/>
+      <c r="M11" s="1"/>
+      <c r="T11" s="1"/>
+    </row>
+    <row r="12" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="3"/>
+      <c r="J12" s="1"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="1"/>
-      <c r="S12" s="1"/>
-    </row>
-    <row r="13" spans="1:19" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L12" s="3"/>
+      <c r="M12" s="1"/>
+      <c r="T12" s="1"/>
+    </row>
+    <row r="13" spans="1:20" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="3"/>
+      <c r="J13" s="1"/>
       <c r="K13" s="3"/>
-      <c r="L13" s="1"/>
-      <c r="S13" s="1"/>
-    </row>
-    <row r="14" spans="1:19" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L13" s="3"/>
+      <c r="M13" s="1"/>
+      <c r="T13" s="1"/>
+    </row>
+    <row r="14" spans="1:20" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="3"/>
+      <c r="J14" s="1"/>
       <c r="K14" s="3"/>
-      <c r="L14" s="1"/>
-      <c r="S14" s="1"/>
-    </row>
-    <row r="15" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L14" s="3"/>
+      <c r="M14" s="1"/>
+      <c r="T14" s="1"/>
+    </row>
+    <row r="15" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="3"/>
+      <c r="J15" s="1"/>
       <c r="K15" s="3"/>
-      <c r="L15" s="1"/>
-      <c r="S15" s="1"/>
-    </row>
-    <row r="16" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L15" s="3"/>
+      <c r="M15" s="1"/>
+      <c r="T15" s="1"/>
+    </row>
+    <row r="16" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="3"/>
+      <c r="J16" s="1"/>
       <c r="K16" s="3"/>
-      <c r="L16" s="1"/>
-      <c r="S16" s="1"/>
-    </row>
-    <row r="17" spans="5:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="3"/>
+      <c r="M16" s="1"/>
+      <c r="T16" s="1"/>
+    </row>
+    <row r="17" spans="5:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="3"/>
+      <c r="J17" s="1"/>
       <c r="K17" s="3"/>
-      <c r="L17" s="1"/>
-      <c r="S17" s="1"/>
-    </row>
-    <row r="18" spans="5:19" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L17" s="3"/>
+      <c r="M17" s="1"/>
+      <c r="T17" s="1"/>
+    </row>
+    <row r="18" spans="5:20" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="3"/>
+      <c r="J18" s="1"/>
       <c r="K18" s="3"/>
-      <c r="L18" s="1"/>
-      <c r="S18" s="1"/>
-    </row>
-    <row r="19" spans="5:19" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L18" s="3"/>
+      <c r="M18" s="1"/>
+      <c r="T18" s="1"/>
+    </row>
+    <row r="19" spans="5:20" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="3"/>
+      <c r="J19" s="1"/>
       <c r="K19" s="3"/>
-      <c r="L19" s="1"/>
-      <c r="S19" s="1"/>
-    </row>
-    <row r="20" spans="5:19" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L19" s="3"/>
+      <c r="M19" s="1"/>
+      <c r="T19" s="1"/>
+    </row>
+    <row r="20" spans="5:20" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="3"/>
+      <c r="J20" s="1"/>
       <c r="K20" s="3"/>
-      <c r="L20" s="1"/>
-      <c r="S20" s="1"/>
-    </row>
-    <row r="21" spans="5:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L20" s="3"/>
+      <c r="M20" s="1"/>
+      <c r="T20" s="1"/>
+    </row>
+    <row r="21" spans="5:20" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="3"/>
+      <c r="J21" s="1"/>
       <c r="K21" s="3"/>
-      <c r="L21" s="1"/>
-      <c r="S21" s="1"/>
-    </row>
-    <row r="22" spans="5:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L21" s="3"/>
+      <c r="M21" s="1"/>
+      <c r="T21" s="1"/>
+    </row>
+    <row r="22" spans="5:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="3"/>
+      <c r="J22" s="1"/>
       <c r="K22" s="3"/>
-      <c r="L22" s="1"/>
-      <c r="S22" s="1"/>
-    </row>
-    <row r="23" spans="5:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L22" s="3"/>
+      <c r="M22" s="1"/>
+      <c r="T22" s="1"/>
+    </row>
+    <row r="23" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="3"/>
+      <c r="J23" s="1"/>
       <c r="K23" s="3"/>
-      <c r="L23" s="1"/>
-      <c r="S23" s="1"/>
-    </row>
-    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="L23" s="3"/>
+      <c r="M23" s="1"/>
+      <c r="T23" s="1"/>
+    </row>
+    <row r="24" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="3"/>
+      <c r="J24" s="1"/>
       <c r="K24" s="3"/>
-      <c r="L24" s="1"/>
-      <c r="Q24" s="1"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="1"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
-    </row>
-    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T24" s="1"/>
+    </row>
+    <row r="25" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="3"/>
+      <c r="J25" s="1"/>
       <c r="K25" s="3"/>
-      <c r="L25" s="1"/>
-      <c r="Q25" s="1"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="1"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
-    </row>
-    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T25" s="1"/>
+    </row>
+    <row r="26" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="3"/>
+      <c r="J26" s="1"/>
       <c r="K26" s="3"/>
-      <c r="L26" s="1"/>
-      <c r="Q26" s="1"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="1"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
-    </row>
-    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T26" s="1"/>
+    </row>
+    <row r="27" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="3"/>
+      <c r="J27" s="1"/>
       <c r="K27" s="3"/>
-      <c r="L27" s="1"/>
-      <c r="Q27" s="1"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="1"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
-    </row>
-    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T27" s="1"/>
+    </row>
+    <row r="28" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="3"/>
+      <c r="J28" s="1"/>
       <c r="K28" s="3"/>
-      <c r="L28" s="1"/>
-      <c r="Q28" s="1"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="1"/>
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
-    </row>
-    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T28" s="1"/>
+    </row>
+    <row r="29" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="3"/>
+      <c r="J29" s="1"/>
       <c r="K29" s="3"/>
-      <c r="L29" s="1"/>
-      <c r="Q29" s="1"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="1"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
-    </row>
-    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T29" s="1"/>
+    </row>
+    <row r="30" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="3"/>
+      <c r="J30" s="1"/>
       <c r="K30" s="3"/>
-      <c r="L30" s="1"/>
-      <c r="Q30" s="1"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="1"/>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
-    </row>
-    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T30" s="1"/>
+    </row>
+    <row r="31" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="3"/>
+      <c r="J31" s="1"/>
       <c r="K31" s="3"/>
-      <c r="L31" s="1"/>
-      <c r="Q31" s="1"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="1"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
-    </row>
-    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T31" s="1"/>
+    </row>
+    <row r="32" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="3"/>
+      <c r="J32" s="1"/>
       <c r="K32" s="3"/>
-      <c r="L32" s="1"/>
-      <c r="Q32" s="1"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="1"/>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
-    </row>
-    <row r="33" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T32" s="1"/>
+    </row>
+    <row r="33" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="3"/>
+      <c r="J33" s="1"/>
       <c r="K33" s="3"/>
-      <c r="L33" s="1"/>
-      <c r="Q33" s="1"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="1"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
-    </row>
-    <row r="34" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T33" s="1"/>
+    </row>
+    <row r="34" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="3"/>
+      <c r="J34" s="1"/>
       <c r="K34" s="3"/>
-      <c r="L34" s="1"/>
-      <c r="Q34" s="1"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="1"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
-    </row>
-    <row r="35" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T34" s="1"/>
+    </row>
+    <row r="35" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
-      <c r="J35" s="3"/>
+      <c r="J35" s="1"/>
       <c r="K35" s="3"/>
-      <c r="L35" s="1"/>
-      <c r="Q35" s="1"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="1"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
-    </row>
-    <row r="36" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T35" s="1"/>
+    </row>
+    <row r="36" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
-      <c r="J36" s="3"/>
+      <c r="J36" s="1"/>
       <c r="K36" s="3"/>
-      <c r="L36" s="1"/>
-      <c r="Q36" s="1"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="1"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
-    </row>
-    <row r="37" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T36" s="1"/>
+    </row>
+    <row r="37" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="3"/>
+      <c r="J37" s="1"/>
       <c r="K37" s="3"/>
-      <c r="L37" s="1"/>
-      <c r="Q37" s="1"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="1"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
-    </row>
-    <row r="38" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T37" s="1"/>
+    </row>
+    <row r="38" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="3"/>
+      <c r="J38" s="1"/>
       <c r="K38" s="3"/>
-      <c r="L38" s="1"/>
-      <c r="Q38" s="1"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="1"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
-    </row>
-    <row r="39" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T38" s="1"/>
+    </row>
+    <row r="39" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="3"/>
+      <c r="J39" s="1"/>
       <c r="K39" s="3"/>
-      <c r="L39" s="1"/>
-      <c r="Q39" s="1"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="1"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
-    </row>
-    <row r="40" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T39" s="1"/>
+    </row>
+    <row r="40" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="3"/>
+      <c r="J40" s="1"/>
       <c r="K40" s="3"/>
-      <c r="L40" s="1"/>
-      <c r="Q40" s="1"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="1"/>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
-    </row>
-    <row r="41" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T40" s="1"/>
+    </row>
+    <row r="41" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="3"/>
+      <c r="J41" s="1"/>
       <c r="K41" s="3"/>
-      <c r="L41" s="1"/>
-      <c r="Q41" s="1"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
-    </row>
-    <row r="42" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T41" s="1"/>
+    </row>
+    <row r="42" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
-      <c r="J42" s="3"/>
+      <c r="J42" s="1"/>
       <c r="K42" s="3"/>
-      <c r="L42" s="1"/>
-      <c r="Q42" s="1"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="1"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
-    </row>
-    <row r="43" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T42" s="1"/>
+    </row>
+    <row r="43" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
-      <c r="J43" s="3"/>
+      <c r="J43" s="1"/>
       <c r="K43" s="3"/>
-      <c r="L43" s="1"/>
-      <c r="Q43" s="1"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="1"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
-    </row>
-    <row r="44" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T43" s="1"/>
+    </row>
+    <row r="44" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
-      <c r="J44" s="3"/>
+      <c r="J44" s="1"/>
       <c r="K44" s="3"/>
-      <c r="L44" s="1"/>
-      <c r="Q44" s="1"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="1"/>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
-    </row>
-    <row r="45" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T44" s="1"/>
+    </row>
+    <row r="45" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
-      <c r="J45" s="3"/>
+      <c r="J45" s="1"/>
       <c r="K45" s="3"/>
-      <c r="L45" s="1"/>
-      <c r="Q45" s="1"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="1"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
-    </row>
-    <row r="46" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T45" s="1"/>
+    </row>
+    <row r="46" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
-      <c r="J46" s="3"/>
+      <c r="J46" s="1"/>
       <c r="K46" s="3"/>
-      <c r="L46" s="1"/>
-      <c r="Q46" s="1"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="1"/>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
-    </row>
-    <row r="47" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="T46" s="1"/>
+    </row>
+    <row r="47" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
-      <c r="J47" s="3"/>
+      <c r="J47" s="1"/>
       <c r="K47" s="3"/>
-      <c r="L47" s="1"/>
-      <c r="Q47" s="1"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="1"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
+      <c r="T47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>